<commit_message>
Added change on dataset currency
</commit_message>
<xml_diff>
--- a/sme-finance-copilot/examples/pos-reports/sample-pos-sales.xlsx
+++ b/sme-finance-copilot/examples/pos-reports/sample-pos-sales.xlsx
@@ -62,12 +62,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>78.90</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -87,7 +87,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>XLSX-1</t>
+          <t>CNY-XLSX-001</t>
         </is>
       </c>
     </row>

</xml_diff>